<commit_message>
board pre production calculate price
</commit_message>
<xml_diff>
--- a/public/demo-files/demo-plates.xlsx
+++ b/public/demo-files/demo-plates.xlsx
@@ -20,9 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production Cost</t>
   </si>
   <si>
     <t xml:space="preserve">Gloss</t>
@@ -116,13 +119,21 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -146,77 +157,89 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.53"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
+      <c r="A4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
+      <c r="A5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
+      <c r="A6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
+      <c r="A7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
+      <c r="A8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
+      <c r="A9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
+      <c r="A10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
+      <c r="A11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
+      <c r="A12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
+      <c r="A13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
+      <c r="A14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
+      <c r="A15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
+      <c r="A16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
+      <c r="A17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
+      <c r="A18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
+      <c r="A19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
+      <c r="A20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
+      <c r="A21" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>